<commit_message>
Replace the repository with the finished monitoring product.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Демо/demo_schedule_timelapse.xlsx
+++ b/Демо/demo_schedule_timelapse.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="timelapse_photos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="methodology" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="timelapse_photos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="methodology" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,13 +436,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,16 +460,11 @@
           <t>date_to</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>zone</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>clearing</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,41 +474,31 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Котлован / нулевой цикл</t>
+          <t>2025-02-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>excavation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-02-20</t>
+          <t>2025-02-10</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>2025-04-20</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Свайное поле</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>foundations</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -524,34 +508,41 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-10-31</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Каркас / плиты перекрытий</t>
+          <t>2025-06-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>superstructure</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-05-01</t>
+          <t>2025-05-20</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Монтаж / крановые работы</t>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>landscaping</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2025-11-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
         </is>
       </c>
     </row>
@@ -620,17 +611,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>clearing</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Земляные работы / котлован</t>
+          <t>Расчистка участка</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>excavator, bulldozer, dump_truck/truck, loader, roller</t>
+          <t>bulldozer/loader, dump_truck/truck</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -650,17 +641,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>clearing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Земляные работы / котлован</t>
+          <t>Расчистка участка</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>excavator, bulldozer, dump_truck/truck, loader, roller</t>
+          <t>bulldozer/loader, dump_truck/truck</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -680,17 +671,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>clearing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Земляные работы / котлован</t>
+          <t>Расчистка участка</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>excavator, bulldozer, dump_truck/truck, loader, roller</t>
+          <t>bulldozer/loader, dump_truck/truck</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -710,17 +701,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>clearing</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Земляные работы / котлован</t>
+          <t>Расчистка участка</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>excavator, bulldozer, dump_truck/truck, loader, roller</t>
+          <t>bulldozer/loader, dump_truck/truck</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -740,17 +731,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>excavation</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Земляные работы / котлован</t>
+          <t>Откопка котлована</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>excavator, bulldozer, dump_truck/truck, loader, roller</t>
+          <t>excavator, dump_truck/truck</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -770,17 +761,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>excavation</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Откопка котлована</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>pile_driver, autocrane/crane_manipulator</t>
+          <t>excavator, dump_truck/truck</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -800,17 +791,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>excavation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Откопка котлована</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>pile_driver, autocrane/crane_manipulator</t>
+          <t>excavator, dump_truck/truck</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -830,17 +821,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>excavation</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Откопка котлована</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>pile_driver, autocrane/crane_manipulator</t>
+          <t>excavator, dump_truck/truck</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -860,17 +851,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>excavation</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Откопка котлована</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>pile_driver, autocrane/crane_manipulator</t>
+          <t>excavator, dump_truck/truck</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -890,12 +881,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>foundations</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Устройство фундаментов</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -920,12 +911,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>piling</t>
+          <t>foundations</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Устройство фундаментов</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -950,17 +941,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>foundations</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Устройство фундаментов</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>pile_driver, autocrane/crane_manipulator</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -980,17 +971,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>foundations</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Устройство фундаментов</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>pile_driver, autocrane/crane_manipulator</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1010,17 +1001,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1040,17 +1031,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1070,17 +1061,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1100,17 +1091,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1130,17 +1121,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1160,17 +1151,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1190,17 +1181,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1220,17 +1211,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1250,17 +1241,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1280,17 +1271,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1310,17 +1301,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1340,17 +1331,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1370,17 +1361,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1400,17 +1391,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1430,17 +1421,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1460,17 +1451,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1490,17 +1481,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>monolith</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>concrete_mixer, concrete_pump, tower_crane</t>
+          <t>tower_crane, concrete_mixer, concrete_pump</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1520,17 +1511,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>superstructure</t>
+          <t>landscaping</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Надземная часть / монтаж</t>
+          <t>Благоустройство</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>tower_crane, autocrane, crane_manipulator</t>
+          <t>roller</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1550,17 +1541,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>superstructure</t>
+          <t>landscaping</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Надземная часть / монтаж</t>
+          <t>Благоустройство</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>tower_crane, autocrane, crane_manipulator</t>
+          <t>roller</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1580,17 +1571,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>superstructure</t>
+          <t>landscaping</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Надземная часть / монтаж</t>
+          <t>Благоустройство</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>tower_crane, autocrane, crane_manipulator</t>
+          <t>roller</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1610,17 +1601,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>superstructure</t>
+          <t>landscaping</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Надземная часть / монтаж</t>
+          <t>Благоустройство</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>tower_crane, autocrane, crane_manipulator</t>
+          <t>roller</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1640,17 +1631,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>superstructure</t>
+          <t>landscaping</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Надземная часть / монтаж</t>
+          <t>Благоустройство</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>tower_crane, autocrane, crane_manipulator</t>
+          <t>roller</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1668,13 +1659,21 @@
           <t>2025-12-26</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>landscaping</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>вне активных этапов</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+          <t>Благоустройство</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>roller</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>Снимок #36, шаг 10 дн.</t>
@@ -1692,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1778,62 +1777,74 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Земляные работы / котлован</t>
+          <t>Расчистка участка</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>1,5–2,5 мес · 2025-01-10 → 2025-03-20</t>
+          <t>1–1,5 мес · 2025-01-10 → 2025-02-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Свайный фундамент</t>
+          <t>Откопка котлована</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>1–2 мес · 2025-02-20 → 2025-04-20</t>
+          <t>1,5–2,5 мес · 2025-02-10 → 2025-04-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Монолитные работы</t>
+          <t>Устройство фундаментов</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>5–8 мес · 2025-04-01 → 2025-10-31</t>
+          <t>1–2 мес · 2025-04-01 → 2025-06-10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Надземная часть / монтаж</t>
+          <t>Монтаж каркаса, стены и перекрытия</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>параллельно монолиту + 1–2 мес мес · 2025-05-01 → 2025-12-20</t>
+          <t>5–8 мес · 2025-05-20 → 2025-11-20</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Благоустройство</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>1–2 мес · 2025-11-01 → 2025-12-30</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Как использовать в Демо</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Лист plan → загрузить как календарный план; снимки именовать по порядку; базовая дата = 2025-01-10, шаг = 10</t>
         </is>

</xml_diff>